<commit_message>
Rodantes: cuerpo = largo entre cabezales (planos Fadesa G690 493 y G689 640)
El modelo restaba el cabezal inferior al cuerpo (25 kg 406, 50 kg 535): los
recipientes salían cortos, livianos y con menos volumen que el del plano.
Ahora 25 kg 493 / 50 kg 640 / 70 kg 798 / 100 kg 917 (volumen 34,4 / 61,8 /
86 / 123 dm³; masa 15,5 / 23,0 / 44,7 / 56,6 kg; Fadesa 15,92 / 23,3).
Recorte de chapa 70 y 100 kg según plano (798 × 1085 y 917 × 1210, 3 por
hoja) con nota de recotizar. Regenerados planos 25-100 kg y AFFF 50 l,
cilindros, despieces, sustitutos, BOM y MRP.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/mrp/MRP_MP.xlsx
+++ b/salida/mrp/MRP_MP.xlsx
@@ -97,17 +97,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FF8B8B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF8B8B"/>
       </patternFill>
     </fill>
   </fills>
@@ -5093,7 +5093,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>3.764</v>
+        <v>3.914</v>
       </c>
       <c r="C9" s="16">
         <f>$B9*'Demanda'!B10</f>
@@ -5143,7 +5143,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4.7</v>
+        <v>4.879</v>
       </c>
       <c r="C10" s="16">
         <f>$B10*'Demanda'!B11</f>
@@ -5193,7 +5193,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>5.264</v>
+        <v>5.457</v>
       </c>
       <c r="C11" s="16">
         <f>$B11*'Demanda'!B12</f>
@@ -5243,7 +5243,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>5.857</v>
+        <v>6.071</v>
       </c>
       <c r="C12" s="16">
         <f>$B12*'Demanda'!B13</f>
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>3.764</v>
+        <v>3.914</v>
       </c>
       <c r="C17" s="16">
         <f>$B17*'Demanda'!B31</f>
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>4.7</v>
+        <v>4.879</v>
       </c>
       <c r="C18" s="16">
         <f>$B18*'Demanda'!B32</f>
@@ -5593,7 +5593,7 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>5.264</v>
+        <v>5.457</v>
       </c>
       <c r="C19" s="16">
         <f>$B19*'Demanda'!B33</f>
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>5.857</v>
+        <v>6.071</v>
       </c>
       <c r="C20" s="16">
         <f>$B20*'Demanda'!B34</f>
@@ -9416,7 +9416,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.144 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.107 de largo desarrollado</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -9483,7 +9483,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.393 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.400 de largo desarrollado</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -9550,7 +9550,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.603 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.674 de largo desarrollado</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 224 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.915 de largo desarrollado</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -9684,7 +9684,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 298 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 224 de largo desarrollado</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -9751,7 +9751,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 458 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 298 de largo desarrollado</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -9818,7 +9818,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 895 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 458 de largo desarrollado</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -22379,27 +22379,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>Chapa LAC 1500 × 3000 e=4,75</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="23" t="inlineStr">
         <is>
           <t>Pradecon S.A.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -22445,10 +22445,10 @@
         <v/>
       </c>
       <c r="AQ20" s="22" t="n">
-        <v>41.925</v>
+        <v>55.953</v>
       </c>
       <c r="AR20" s="22" t="n">
-        <v>55.947</v>
+        <v>55.91</v>
       </c>
     </row>
     <row r="21">
@@ -23152,27 +23152,27 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>Planchuela SAE 1010 30 × 3</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>barra 6 m</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C31" s="24" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D31" s="24" t="inlineStr">
         <is>
           <t>Hierros Parrotta</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E31" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -23231,27 +23231,27 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>Planchuela SAE 1010 40 × 4</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>barra 6 m</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>Hierros Parrotta</t>
         </is>
       </c>
-      <c r="E32" s="23" t="inlineStr">
+      <c r="E32" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -23304,27 +23304,27 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="inlineStr">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>Recorte de chapa LAC e=3,2 para el apoyo plegado</t>
         </is>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr">
+      <c r="D33" s="24" t="inlineStr">
         <is>
           <t>Pradecon S.A.</t>
         </is>
       </c>
-      <c r="E33" s="23" t="inlineStr">
+      <c r="E33" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -23462,27 +23462,27 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>Redondo liso SAE 1010 Ø8</t>
         </is>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="24" t="inlineStr">
         <is>
           <t>barra 6 m</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D35" s="23" t="inlineStr">
+      <c r="D35" s="24" t="inlineStr">
         <is>
           <t>Hierros Parrotta</t>
         </is>
       </c>
-      <c r="E35" s="23" t="inlineStr">
+      <c r="E35" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -23528,10 +23528,10 @@
         <v/>
       </c>
       <c r="AQ35" s="22" t="n">
-        <v>0.1089</v>
+        <v>0.128</v>
       </c>
       <c r="AR35" s="22" t="n">
-        <v>0.1265</v>
+        <v>0.1478</v>
       </c>
     </row>
     <row r="36">
@@ -25028,7 +25028,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.144 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.107 de largo desarrollado</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -25091,14 +25091,14 @@
         <f>SUMPRODUCT($AK57:$AR57,$AK$14:$AR$14)*IF($E57="CABA",'Parametros'!K$7,IF($E57="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AP57" s="22" t="n">
+      <c r="AO57" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.393 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.400 de largo desarrollado</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -25161,14 +25161,14 @@
         <f>SUMPRODUCT($AK58:$AR58,$AK$14:$AR$14)*IF($E58="CABA",'Parametros'!K$7,IF($E58="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AQ58" s="22" t="n">
+      <c r="AP58" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.603 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.674 de largo desarrollado</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -25231,14 +25231,14 @@
         <f>SUMPRODUCT($AK59:$AR59,$AK$14:$AR$14)*IF($E59="CABA",'Parametros'!K$7,IF($E59="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AR59" s="22" t="n">
+      <c r="AQ59" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 224 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.915 de largo desarrollado</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -25301,14 +25301,14 @@
         <f>SUMPRODUCT($AK60:$AR60,$AK$14:$AR$14)*IF($E60="CABA",'Parametros'!K$7,IF($E60="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AL60" s="22" t="n">
+      <c r="AR60" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 298 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 224 de largo desarrollado</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -25371,14 +25371,14 @@
         <f>SUMPRODUCT($AK61:$AR61,$AK$14:$AR$14)*IF($E61="CABA",'Parametros'!K$7,IF($E61="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AM61" s="22" t="n">
+      <c r="AL61" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 458 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 298 de largo desarrollado</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -25441,14 +25441,14 @@
         <f>SUMPRODUCT($AK62:$AR62,$AK$14:$AR$14)*IF($E62="CABA",'Parametros'!K$7,IF($E62="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AN62" s="22" t="n">
+      <c r="AM62" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 895 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 458 de largo desarrollado</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -25511,32 +25511,32 @@
         <f>SUMPRODUCT($AK63:$AR63,$AK$14:$AR$14)*IF($E63="CABA",'Parametros'!K$7,IF($E63="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AO63" s="22" t="n">
+      <c r="AN63" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="24" t="inlineStr">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>Manómetro — Ø28 esfera, rango 0-3,5 MPa, sector verde en 1,4</t>
         </is>
       </c>
-      <c r="B64" s="24" t="inlineStr">
+      <c r="B64" s="25" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C64" s="24" t="inlineStr">
+      <c r="C64" s="25" t="inlineStr">
         <is>
           <t>Componente comprado</t>
         </is>
       </c>
-      <c r="D64" s="24" t="inlineStr">
+      <c r="D64" s="25" t="inlineStr">
         <is>
           <t>Yukon / MatafuegosYa S.R.L.</t>
         </is>
       </c>
-      <c r="E64" s="24" t="inlineStr">
+      <c r="E64" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -25586,27 +25586,27 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="24" t="inlineStr">
+      <c r="A65" s="25" t="inlineStr">
         <is>
           <t>Manómetro — Ø38 esfera, rango 0-3,5 MPa, sector verde en 1,4</t>
         </is>
       </c>
-      <c r="B65" s="24" t="inlineStr">
+      <c r="B65" s="25" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C65" s="24" t="inlineStr">
+      <c r="C65" s="25" t="inlineStr">
         <is>
           <t>Componente comprado</t>
         </is>
       </c>
-      <c r="D65" s="24" t="inlineStr">
+      <c r="D65" s="25" t="inlineStr">
         <is>
           <t>Yukon / MatafuegosYa S.R.L.</t>
         </is>
       </c>
-      <c r="E65" s="24" t="inlineStr">
+      <c r="E65" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -25662,27 +25662,27 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="24" t="inlineStr">
+      <c r="A66" s="25" t="inlineStr">
         <is>
           <t>Manómetro — Ø50 esfera, rango 0-3,5 MPa, sector verde en 1,4</t>
         </is>
       </c>
-      <c r="B66" s="24" t="inlineStr">
+      <c r="B66" s="25" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C66" s="24" t="inlineStr">
+      <c r="C66" s="25" t="inlineStr">
         <is>
           <t>Componente comprado</t>
         </is>
       </c>
-      <c r="D66" s="24" t="inlineStr">
+      <c r="D66" s="25" t="inlineStr">
         <is>
           <t>Yukon / MatafuegosYa S.R.L.</t>
         </is>
       </c>
-      <c r="E66" s="24" t="inlineStr">
+      <c r="E66" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -25741,27 +25741,27 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="24" t="inlineStr">
+      <c r="A67" s="25" t="inlineStr">
         <is>
           <t>Neumático macizo — Ø300 × 55 de ancho</t>
         </is>
       </c>
-      <c r="B67" s="24" t="inlineStr">
+      <c r="B67" s="25" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C67" s="24" t="inlineStr">
+      <c r="C67" s="25" t="inlineStr">
         <is>
           <t>Componente comprado</t>
         </is>
       </c>
-      <c r="D67" s="24" t="inlineStr">
+      <c r="D67" s="25" t="inlineStr">
         <is>
           <t>Ruedar</t>
         </is>
       </c>
-      <c r="E67" s="24" t="inlineStr">
+      <c r="E67" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -25884,27 +25884,27 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="25" t="inlineStr">
+      <c r="A69" s="23" t="inlineStr">
         <is>
           <t>Neumático macizo — Ø400 × 80 de ancho</t>
         </is>
       </c>
-      <c r="B69" s="25" t="inlineStr">
+      <c r="B69" s="23" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C69" s="25" t="inlineStr">
+      <c r="C69" s="23" t="inlineStr">
         <is>
           <t>Componente comprado</t>
         </is>
       </c>
-      <c r="D69" s="25" t="inlineStr">
+      <c r="D69" s="23" t="inlineStr">
         <is>
           <t>Ruedar</t>
         </is>
       </c>
-      <c r="E69" s="25" t="inlineStr">
+      <c r="E69" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -26915,27 +26915,27 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="23" t="inlineStr">
+      <c r="A83" s="24" t="inlineStr">
         <is>
           <t>Alambre MAG ER70S-6 Ø0,9 (AWS A5.18)</t>
         </is>
       </c>
-      <c r="B83" s="23" t="inlineStr">
+      <c r="B83" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C83" s="23" t="inlineStr">
+      <c r="C83" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D83" s="23" t="inlineStr">
+      <c r="D83" s="24" t="inlineStr">
         <is>
           <t>Conarco (ESAB Argentina)</t>
         </is>
       </c>
-      <c r="E83" s="23" t="inlineStr">
+      <c r="E83" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -26994,27 +26994,27 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="23" t="inlineStr">
+      <c r="A84" s="24" t="inlineStr">
         <is>
           <t>Alambre MAG ER70S-6 Ø1,2 (AWS A5.18)</t>
         </is>
       </c>
-      <c r="B84" s="23" t="inlineStr">
+      <c r="B84" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C84" s="23" t="inlineStr">
+      <c r="C84" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D84" s="23" t="inlineStr">
+      <c r="D84" s="24" t="inlineStr">
         <is>
           <t>Conarco (ESAB Argentina)</t>
         </is>
       </c>
-      <c r="E84" s="23" t="inlineStr">
+      <c r="E84" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -27060,40 +27060,40 @@
         <v/>
       </c>
       <c r="AO84" s="22" t="n">
-        <v>0.3374</v>
+        <v>0.3429</v>
       </c>
       <c r="AP84" s="22" t="n">
-        <v>0.4194</v>
+        <v>0.426</v>
       </c>
       <c r="AQ84" s="22" t="n">
-        <v>0.9806</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="AR84" s="22" t="n">
-        <v>1.0848</v>
+        <v>1.0968</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="23" t="inlineStr">
+      <c r="A85" s="24" t="inlineStr">
         <is>
           <t>Gas de protección MAG Arcal 21 / ARCAL Speed (Ar + 8 % CO₂, M20)</t>
         </is>
       </c>
-      <c r="B85" s="23" t="inlineStr">
+      <c r="B85" s="24" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C85" s="23" t="inlineStr">
+      <c r="C85" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D85" s="23" t="inlineStr">
+      <c r="D85" s="24" t="inlineStr">
         <is>
           <t>Air Liquide Argentina - sucursal Piñeyro</t>
         </is>
       </c>
-      <c r="E85" s="23" t="inlineStr">
+      <c r="E85" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -27151,40 +27151,40 @@
         <v>40.7</v>
       </c>
       <c r="AO85" s="22" t="n">
-        <v>52.7</v>
+        <v>54.8</v>
       </c>
       <c r="AP85" s="22" t="n">
-        <v>65.8</v>
+        <v>68.3</v>
       </c>
       <c r="AQ85" s="22" t="n">
-        <v>73.7</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AR85" s="22" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="25" t="inlineStr">
+      <c r="A86" s="23" t="inlineStr">
         <is>
           <t>Granalla de acero S330 / S390 (ISO 11124-3, SAE J444)</t>
         </is>
       </c>
-      <c r="B86" s="25" t="inlineStr">
+      <c r="B86" s="23" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C86" s="25" t="inlineStr">
+      <c r="C86" s="23" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D86" s="25" t="inlineStr">
+      <c r="D86" s="23" t="inlineStr">
         <is>
           <t>CyM Materiales</t>
         </is>
       </c>
-      <c r="E86" s="25" t="inlineStr">
+      <c r="E86" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -27401,27 +27401,27 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="23" t="inlineStr">
+      <c r="A89" s="24" t="inlineStr">
         <is>
           <t>Gas impulsor: N₂</t>
         </is>
       </c>
-      <c r="B89" s="23" t="inlineStr">
+      <c r="B89" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C89" s="23" t="inlineStr">
+      <c r="C89" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D89" s="23" t="inlineStr">
+      <c r="D89" s="24" t="inlineStr">
         <is>
           <t>Air Liquide Argentina - sucursal Piñeyro</t>
         </is>
       </c>
-      <c r="E89" s="23" t="inlineStr">
+      <c r="E89" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -27492,27 +27492,27 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="23" t="inlineStr">
+      <c r="A90" s="24" t="inlineStr">
         <is>
           <t>Polvo químico seco ABC 60 (Sello IRAM 3569)</t>
         </is>
       </c>
-      <c r="B90" s="23" t="inlineStr">
+      <c r="B90" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C90" s="23" t="inlineStr">
+      <c r="C90" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D90" s="23" t="inlineStr">
+      <c r="D90" s="24" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E90" s="23" t="inlineStr">
+      <c r="E90" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -27571,27 +27571,27 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="23" t="inlineStr">
+      <c r="A91" s="24" t="inlineStr">
         <is>
           <t>Polvo químico seco ABC 90 (Sello IRAM 3569)</t>
         </is>
       </c>
-      <c r="B91" s="23" t="inlineStr">
+      <c r="B91" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C91" s="23" t="inlineStr">
+      <c r="C91" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D91" s="23" t="inlineStr">
+      <c r="D91" s="24" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E91" s="23" t="inlineStr">
+      <c r="E91" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -29255,27 +29255,27 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="23" t="inlineStr">
+      <c r="A113" s="24" t="inlineStr">
         <is>
           <t>Cinta de embalaje PP 48 mm (cierre de la caja)</t>
         </is>
       </c>
-      <c r="B113" s="23" t="inlineStr">
+      <c r="B113" s="24" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C113" s="23" t="inlineStr">
+      <c r="C113" s="24" t="inlineStr">
         <is>
           <t>Embalaje</t>
         </is>
       </c>
-      <c r="D113" s="23" t="inlineStr">
+      <c r="D113" s="24" t="inlineStr">
         <is>
           <t>MV Embalajes</t>
         </is>
       </c>
-      <c r="E113" s="23" t="inlineStr">
+      <c r="E113" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -29583,27 +29583,27 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="23" t="inlineStr">
+      <c r="A117" s="24" t="inlineStr">
         <is>
           <t>Film stretch (fracción del pallet)</t>
         </is>
       </c>
-      <c r="B117" s="23" t="inlineStr">
+      <c r="B117" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C117" s="23" t="inlineStr">
+      <c r="C117" s="24" t="inlineStr">
         <is>
           <t>Embalaje</t>
         </is>
       </c>
-      <c r="D117" s="23" t="inlineStr">
+      <c r="D117" s="24" t="inlineStr">
         <is>
           <t>MV Embalajes</t>
         </is>
       </c>
-      <c r="E117" s="23" t="inlineStr">
+      <c r="E117" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -30848,27 +30848,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Equipo terminado comprado (fabricante con Sello IRAM): FL_MAT_CLASED_9l</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>Equipo terminado comprado</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t>Matafuegos Georgia - venta mayorista</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -31921,27 +31921,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Chapa LAC 1500 × 3000 e=4,75</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>Pradecon S.A.</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -31987,10 +31987,10 @@
         <v/>
       </c>
       <c r="AQ19" s="22" t="n">
-        <v>41.925</v>
+        <v>55.953</v>
       </c>
       <c r="AR19" s="22" t="n">
-        <v>55.947</v>
+        <v>55.91</v>
       </c>
     </row>
     <row r="20">
@@ -32694,27 +32694,27 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A30" s="24" t="inlineStr">
         <is>
           <t>Redondo liso SAE 1010 Ø8</t>
         </is>
       </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>barra 6 m</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>Materia prima</t>
         </is>
       </c>
-      <c r="D30" s="23" t="inlineStr">
+      <c r="D30" s="24" t="inlineStr">
         <is>
           <t>Hierros Parrotta</t>
         </is>
       </c>
-      <c r="E30" s="23" t="inlineStr">
+      <c r="E30" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -32760,10 +32760,10 @@
         <v/>
       </c>
       <c r="AQ30" s="22" t="n">
-        <v>0.1089</v>
+        <v>0.128</v>
       </c>
       <c r="AR30" s="22" t="n">
-        <v>0.1265</v>
+        <v>0.1478</v>
       </c>
     </row>
     <row r="31">
@@ -33753,27 +33753,27 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="inlineStr">
+      <c r="A45" s="24" t="inlineStr">
         <is>
           <t>Alambre MAG ER70S-6 Ø0,9 (AWS A5.18)</t>
         </is>
       </c>
-      <c r="B45" s="23" t="inlineStr">
+      <c r="B45" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C45" s="23" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D45" s="23" t="inlineStr">
+      <c r="D45" s="24" t="inlineStr">
         <is>
           <t>Conarco (ESAB Argentina)</t>
         </is>
       </c>
-      <c r="E45" s="23" t="inlineStr">
+      <c r="E45" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -33832,27 +33832,27 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>Alambre MAG ER70S-6 Ø1,2 (AWS A5.18)</t>
         </is>
       </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C46" s="23" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D46" s="23" t="inlineStr">
+      <c r="D46" s="24" t="inlineStr">
         <is>
           <t>Conarco (ESAB Argentina)</t>
         </is>
       </c>
-      <c r="E46" s="23" t="inlineStr">
+      <c r="E46" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -33898,40 +33898,40 @@
         <v/>
       </c>
       <c r="AO46" s="22" t="n">
-        <v>0.3374</v>
+        <v>0.3429</v>
       </c>
       <c r="AP46" s="22" t="n">
-        <v>0.4194</v>
+        <v>0.426</v>
       </c>
       <c r="AQ46" s="22" t="n">
-        <v>0.9806</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="AR46" s="22" t="n">
-        <v>1.0848</v>
+        <v>1.0968</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="inlineStr">
+      <c r="A47" s="24" t="inlineStr">
         <is>
           <t>Gas de protección MAG Arcal 21 / ARCAL Speed (Ar + 8 % CO₂, M20)</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C47" s="23" t="inlineStr">
+      <c r="C47" s="24" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D47" s="23" t="inlineStr">
+      <c r="D47" s="24" t="inlineStr">
         <is>
           <t>Air Liquide Argentina - sucursal Piñeyro</t>
         </is>
       </c>
-      <c r="E47" s="23" t="inlineStr">
+      <c r="E47" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -33989,40 +33989,40 @@
         <v>40.7</v>
       </c>
       <c r="AO47" s="22" t="n">
-        <v>52.7</v>
+        <v>54.8</v>
       </c>
       <c r="AP47" s="22" t="n">
-        <v>65.8</v>
+        <v>68.3</v>
       </c>
       <c r="AQ47" s="22" t="n">
-        <v>73.7</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AR47" s="22" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="inlineStr">
+      <c r="A48" s="23" t="inlineStr">
         <is>
           <t>Granalla de acero S330 / S390 (ISO 11124-3, SAE J444)</t>
         </is>
       </c>
-      <c r="B48" s="25" t="inlineStr">
+      <c r="B48" s="23" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C48" s="25" t="inlineStr">
+      <c r="C48" s="23" t="inlineStr">
         <is>
           <t>Consumible de proceso</t>
         </is>
       </c>
-      <c r="D48" s="25" t="inlineStr">
+      <c r="D48" s="23" t="inlineStr">
         <is>
           <t>CyM Materiales</t>
         </is>
       </c>
-      <c r="E48" s="25" t="inlineStr">
+      <c r="E48" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -34610,27 +34610,27 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="inlineStr">
+      <c r="A56" s="24" t="inlineStr">
         <is>
           <t>Cinta de embalaje PP 48 mm (cierre de la caja)</t>
         </is>
       </c>
-      <c r="B56" s="23" t="inlineStr">
+      <c r="B56" s="24" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C56" s="23" t="inlineStr">
+      <c r="C56" s="24" t="inlineStr">
         <is>
           <t>Embalaje</t>
         </is>
       </c>
-      <c r="D56" s="23" t="inlineStr">
+      <c r="D56" s="24" t="inlineStr">
         <is>
           <t>MV Embalajes</t>
         </is>
       </c>
-      <c r="E56" s="23" t="inlineStr">
+      <c r="E56" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -34938,27 +34938,27 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="23" t="inlineStr">
+      <c r="A60" s="24" t="inlineStr">
         <is>
           <t>Film stretch (fracción del pallet)</t>
         </is>
       </c>
-      <c r="B60" s="23" t="inlineStr">
+      <c r="B60" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C60" s="23" t="inlineStr">
+      <c r="C60" s="24" t="inlineStr">
         <is>
           <t>Embalaje</t>
         </is>
       </c>
-      <c r="D60" s="23" t="inlineStr">
+      <c r="D60" s="24" t="inlineStr">
         <is>
           <t>MV Embalajes</t>
         </is>
       </c>
-      <c r="E60" s="23" t="inlineStr">
+      <c r="E60" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -35199,27 +35199,27 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="25" t="inlineStr">
+      <c r="A63" s="23" t="inlineStr">
         <is>
           <t>Tapón protector de rosca del cuello</t>
         </is>
       </c>
-      <c r="B63" s="25" t="inlineStr">
+      <c r="B63" s="23" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C63" s="25" t="inlineStr">
+      <c r="C63" s="23" t="inlineStr">
         <is>
           <t>Embalaje</t>
         </is>
       </c>
-      <c r="D63" s="25" t="inlineStr">
+      <c r="D63" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E63" s="25" t="inlineStr">
+      <c r="E63" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -37944,27 +37944,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Gas impulsor: N₂</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>Air Liquide Argentina - sucursal Piñeyro</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -38135,27 +38135,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Polvo químico seco ABC 60 (Sello IRAM 3569)</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E18" s="23" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -38298,27 +38298,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Polvo químico seco ABC 90 (Sello IRAM 3569)</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Carga (agente y gas)</t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E19" s="23" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -38461,27 +38461,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Acetato de potasio - DEMSA Kitchen (IRAM 3697)</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>Polvex S.R.L. / Sancibrao</t>
         </is>
       </c>
-      <c r="E20" s="23" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -38612,27 +38612,27 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Concentrado espumígeno AFFF 3 % (IRAM 3515)</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -39443,27 +39443,27 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>HCFC 123 / HFC 236fa (agente limpio)</t>
         </is>
       </c>
-      <c r="B26" s="25" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C26" s="25" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E26" s="25" t="inlineStr">
+      <c r="E26" s="23" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -39594,27 +39594,27 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="24" t="inlineStr">
         <is>
           <t>Junta tórica de asiento del cuello</t>
         </is>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="24" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D27" s="23" t="inlineStr">
+      <c r="D27" s="24" t="inlineStr">
         <is>
           <t>Argensold</t>
         </is>
       </c>
-      <c r="E27" s="23" t="inlineStr">
+      <c r="E27" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -40239,27 +40239,27 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>Polvo para metales combustibles clase D</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C30" s="25" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D30" s="25" t="inlineStr">
         <is>
           <t>DEM S.A. (DEMSA)</t>
         </is>
       </c>
-      <c r="E30" s="24" t="inlineStr">
+      <c r="E30" s="25" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
@@ -40390,27 +40390,27 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>Polvo químico seco BC (bicarbonato)</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C31" s="24" t="inlineStr">
         <is>
           <t>Recarga y mantenimiento</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D31" s="24" t="inlineStr">
         <is>
           <t>Polvex S.R.L. / Sancibrao</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E31" s="24" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>

</xml_diff>

<commit_message>
Hoja 4 toda a color y carros con accesorios adelante
- Etiqueta R1 como las relevadas: encabezado de marca en el color del agente,
  franja INSTRUCCIONES amarilla con números en rojo, ilustraciones de cada
  paso, símbolos IRAM 3550 5.2.5.3 (K hexágono negro, IRAM 3517-2 7.2.2),
  pictogramas NFPA 10 anexo B con figura, franja de aptitud eléctrica,
  logos, QR y pie.
- Vista R2 coloreada pieza por pieza (z-buffer: sólo lo visible), con la
  etiqueta impresa, manómetro con zonas, oblea, estampilla y tarjeta.
- R4-R8, tabla de contenido, cilindros (FL_REC hoja 3) y sustitutos
  (frente e isometría) a color.
- Carros: eje, manija y etiqueta atrás; ganchos, manga enrollada, tobera
  y tercera pata adelante. Pata 80 x 60 / 100 x 80 de 3,2 mm (puesto 2).
  Marcado en el puesto 11; ruta, alambre Ø1,0 y despiece según el proceso.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/mrp/MRP_MP.xlsx
+++ b/salida/mrp/MRP_MP.xlsx
@@ -8813,7 +8813,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 1.043 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.037 de largo desarrollado</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -8880,7 +8880,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 1.339 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.305 de largo desarrollado</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -8947,7 +8947,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 671 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.371 de largo desarrollado</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -9014,7 +9014,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 892 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.714 de largo desarrollado</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -9081,7 +9081,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.045 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.698 de largo desarrollado</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -9148,7 +9148,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 238 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.168 de largo desarrollado</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -9215,7 +9215,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 329 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.398 de largo desarrollado</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -9282,7 +9282,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 518 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.871 de largo desarrollado</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -9349,7 +9349,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 647 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 238 de largo desarrollado</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -9416,7 +9416,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 839 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 329 de largo desarrollado</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -9483,7 +9483,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 991 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 518 de largo desarrollado</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -11024,7 +11024,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Alambre MAG ER70S-6 Ø1,2 (AWS A5.18)</t>
+          <t>Alambre MAG ER70S-6 Ø1,0 (AWS A5.18)</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -11627,7 +11627,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 168 × 136 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 168 × 137 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -11694,7 +11694,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 234 × 151 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 234 × 152 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -11761,7 +11761,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 289 × 142 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 289 × 144 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -11828,7 +11828,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 343 × 221 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 343 × 224 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -11895,7 +11895,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 522 × 208 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 522 × 210 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -11962,7 +11962,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 604 × 204 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 604 × 207 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -12029,7 +12029,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 736 × 211 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 736 × 214 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -21754,16 +21754,16 @@
         <v/>
       </c>
       <c r="AO17" s="22" t="n">
-        <v>0.2797</v>
+        <v>0.2216</v>
       </c>
       <c r="AP17" s="22" t="n">
-        <v>0.2789</v>
+        <v>0.219</v>
       </c>
       <c r="AQ17" s="22" t="n">
-        <v>0.3184</v>
+        <v>0.2566</v>
       </c>
       <c r="AR17" s="22" t="n">
-        <v>0.3021</v>
+        <v>0.2366</v>
       </c>
     </row>
     <row r="18">
@@ -23920,7 +23920,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 1.043 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.037 de largo desarrollado</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -23983,14 +23983,14 @@
         <f>SUMPRODUCT($AK48:$AR48,$AK$14:$AR$14)*IF($E48="CABA",'Parametros'!K$7,IF($E48="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AQ48" s="22" t="n">
+      <c r="AO48" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 1.339 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.305 de largo desarrollado</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -24053,14 +24053,14 @@
         <f>SUMPRODUCT($AK49:$AR49,$AK$14:$AR$14)*IF($E49="CABA",'Parametros'!K$7,IF($E49="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AR49" s="22" t="n">
+      <c r="AP49" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 671 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.371 de largo desarrollado</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -24123,14 +24123,14 @@
         <f>SUMPRODUCT($AK50:$AR50,$AK$14:$AR$14)*IF($E50="CABA",'Parametros'!K$7,IF($E50="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AO50" s="22" t="n">
+      <c r="AQ50" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Manguera (tramo enrollado) — Ø25 × 892 de largo desarrollado</t>
+          <t>Manguera (tramo enrollado) — Ø25 × 1.714 de largo desarrollado</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -24193,14 +24193,14 @@
         <f>SUMPRODUCT($AK51:$AR51,$AK$14:$AR$14)*IF($E51="CABA",'Parametros'!K$7,IF($E51="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AP51" s="22" t="n">
+      <c r="AR51" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 1.045 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 1.698 de largo desarrollado</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -24263,14 +24263,14 @@
         <f>SUMPRODUCT($AK52:$AR52,$AK$14:$AR$14)*IF($E52="CABA",'Parametros'!K$7,IF($E52="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AR52" s="22" t="n">
+      <c r="AO52" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 238 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.168 de largo desarrollado</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -24333,14 +24333,14 @@
         <f>SUMPRODUCT($AK53:$AR53,$AK$14:$AR$14)*IF($E53="CABA",'Parametros'!K$7,IF($E53="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AL53" s="22" t="n">
+      <c r="AP53" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 329 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.398 de largo desarrollado</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -24403,14 +24403,14 @@
         <f>SUMPRODUCT($AK54:$AR54,$AK$14:$AR$14)*IF($E54="CABA",'Parametros'!K$7,IF($E54="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AM54" s="22" t="n">
+      <c r="AQ54" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 518 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 2.871 de largo desarrollado</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -24473,14 +24473,14 @@
         <f>SUMPRODUCT($AK55:$AR55,$AK$14:$AR$14)*IF($E55="CABA",'Parametros'!K$7,IF($E55="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AN55" s="22" t="n">
+      <c r="AR55" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 647 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 238 de largo desarrollado</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -24543,14 +24543,14 @@
         <f>SUMPRODUCT($AK56:$AR56,$AK$14:$AR$14)*IF($E56="CABA",'Parametros'!K$7,IF($E56="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AO56" s="22" t="n">
+      <c r="AL56" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 839 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 329 de largo desarrollado</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -24613,14 +24613,14 @@
         <f>SUMPRODUCT($AK57:$AR57,$AK$14:$AR$14)*IF($E57="CABA",'Parametros'!K$7,IF($E57="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AP57" s="22" t="n">
+      <c r="AM57" s="22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Manguera — Ø16 × 991 de largo desarrollado</t>
+          <t>Manguera — Ø16 × 518 de largo desarrollado</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -24683,7 +24683,7 @@
         <f>SUMPRODUCT($AK58:$AR58,$AK$14:$AR$14)*IF($E58="CABA",'Parametros'!K$7,IF($E58="PBA",1-'Parametros'!K$7,1))</f>
         <v/>
       </c>
-      <c r="AQ58" s="22" t="n">
+      <c r="AN58" s="22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -26101,7 +26101,7 @@
     <row r="78">
       <c r="A78" s="23" t="inlineStr">
         <is>
-          <t>Alambre MAG ER70S-6 Ø1,2 (AWS A5.18)</t>
+          <t>Alambre MAG ER70S-6 Ø1,0 (AWS A5.18)</t>
         </is>
       </c>
       <c r="B78" s="23" t="inlineStr">
@@ -26848,7 +26848,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 168 × 136 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 168 × 137 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -26918,7 +26918,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 234 × 151 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 234 × 152 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -26988,7 +26988,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 289 × 142 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 289 × 144 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -27058,7 +27058,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 343 × 221 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 343 × 224 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -27128,7 +27128,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 522 × 208 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 522 × 210 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -27198,7 +27198,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 604 × 204 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 604 × 207 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -27268,7 +27268,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Etiqueta / placa de características — 736 × 211 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
+          <t>Etiqueta / placa de características — 736 × 214 (desarrollo × alto: panel central 108° + 2 alas laterales), e ≈ 0,3, laminado UV</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -32665,7 +32665,7 @@
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>Alambre MAG ER70S-6 Ø1,2 (AWS A5.18)</t>
+          <t>Alambre MAG ER70S-6 Ø1,0 (AWS A5.18)</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">

</xml_diff>